<commit_message>
Empiezo a escribir el TFM
</commit_message>
<xml_diff>
--- a/modelado/modelos/resultados/Class/BL_cla.xlsx
+++ b/modelado/modelos/resultados/Class/BL_cla.xlsx
@@ -169,7 +169,62 @@
       <row>0</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="8096250" cy="2990850"/>
+    <ext cx="8096250" cy="3000375"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>13</col>
+      <colOff>0</colOff>
+      <row>20</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="6296025" cy="4667250"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="2" name="Image 2" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>13</col>
+      <colOff>0</colOff>
+      <row>0</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="8096250" cy="3000375"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -214,61 +269,6 @@
         <a:ln>
           <a:prstDash val="solid"/>
         </a:ln>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-</wsDr>
-</file>
-
-<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <oneCellAnchor>
-    <from>
-      <col>13</col>
-      <colOff>0</colOff>
-      <row>0</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="8096250" cy="2990850"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="1" name="Image 1" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId1"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>13</col>
-      <colOff>0</colOff>
-      <row>20</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="6296025" cy="4667250"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="2" name="Image 2" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId2"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>

</xml_diff>

<commit_message>
Se ha añadido más datos (desde 2009-2025)
</commit_message>
<xml_diff>
--- a/modelado/modelos/resultados/Class/BL_cla.xlsx
+++ b/modelado/modelos/resultados/Class/BL_cla.xlsx
@@ -183,61 +183,6 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>13</col>
-      <colOff>0</colOff>
-      <row>20</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="6296025" cy="4667250"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="2" name="Image 2" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId2"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-</wsDr>
-</file>
-
-<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <oneCellAnchor>
-    <from>
-      <col>13</col>
-      <colOff>0</colOff>
-      <row>0</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="8096250" cy="3000375"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="1" name="Image 1" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId1"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
         <a:ln>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -269,6 +214,61 @@
         <a:ln>
           <a:prstDash val="solid"/>
         </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>13</col>
+      <colOff>0</colOff>
+      <row>0</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="8096250" cy="3000375"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>13</col>
+      <colOff>0</colOff>
+      <row>20</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="6296025" cy="4667250"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="2" name="Image 2" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -588,16 +588,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.7664520743919886</v>
+        <v>0.8004422332780542</v>
       </c>
       <c r="C3" t="n">
-        <v>0.8862696443341604</v>
+        <v>0.9532587228439763</v>
       </c>
       <c r="D3" t="n">
-        <v>0.822017644802455</v>
+        <v>0.8701923076923077</v>
       </c>
       <c r="E3" t="n">
-        <v>2418</v>
+        <v>3038</v>
       </c>
     </row>
     <row r="4">
@@ -607,16 +607,16 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.7607655502392344</v>
+        <v>0.7123287671232876</v>
       </c>
       <c r="C4" t="n">
-        <v>0.6643454038997214</v>
+        <v>0.426812585499316</v>
       </c>
       <c r="D4" t="n">
-        <v>0.7092936802973978</v>
+        <v>0.5337895637296834</v>
       </c>
       <c r="E4" t="n">
-        <v>1436</v>
+        <v>731</v>
       </c>
     </row>
     <row r="5">
@@ -626,16 +626,16 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.7422222222222222</v>
+        <v>0.7680180180180181</v>
       </c>
       <c r="C5" t="n">
-        <v>0.5170278637770898</v>
+        <v>0.466484268125855</v>
       </c>
       <c r="D5" t="n">
-        <v>0.6094890510948905</v>
+        <v>0.5804255319148937</v>
       </c>
       <c r="E5" t="n">
-        <v>646</v>
+        <v>731</v>
       </c>
     </row>
     <row r="6">
@@ -645,16 +645,16 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.7624444444444445</v>
+        <v>0.7886666666666666</v>
       </c>
       <c r="C6" t="n">
-        <v>0.7624444444444445</v>
+        <v>0.7886666666666666</v>
       </c>
       <c r="D6" t="n">
-        <v>0.7624444444444445</v>
+        <v>0.7886666666666666</v>
       </c>
       <c r="E6" t="n">
-        <v>0.7624444444444445</v>
+        <v>0.7886666666666666</v>
       </c>
     </row>
     <row r="7">
@@ -664,13 +664,13 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.7564799489511485</v>
+        <v>0.7602630061397866</v>
       </c>
       <c r="C7" t="n">
-        <v>0.6892143040036572</v>
+        <v>0.6155185254897158</v>
       </c>
       <c r="D7" t="n">
-        <v>0.7136001253982478</v>
+        <v>0.6614691344456283</v>
       </c>
       <c r="E7" t="n">
         <v>4500</v>
@@ -683,13 +683,13 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.7611591114619833</v>
+        <v>0.7808615565860051</v>
       </c>
       <c r="C8" t="n">
-        <v>0.7624444444444445</v>
+        <v>0.7886666666666666</v>
       </c>
       <c r="D8" t="n">
-        <v>0.7555365148992663</v>
+        <v>0.7684745479300926</v>
       </c>
       <c r="E8" t="n">
         <v>4500</v>
@@ -709,7 +709,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.6978183002279388</v>
+        <v>0.7702127659574468</v>
       </c>
     </row>
     <row r="12">
@@ -719,7 +719,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.5495391705069125</v>
+        <v>0.3640606767794632</v>
       </c>
     </row>
     <row r="13">
@@ -729,7 +729,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.4383202099737533</v>
+        <v>0.4088729016786571</v>
       </c>
     </row>
     <row r="16">
@@ -746,10 +746,10 @@
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>0.5779459033773803</v>
+        <v>0.5031794425997246</v>
       </c>
       <c r="B17" t="n">
-        <v>0.2739458807739117</v>
+        <v>0.4482800819931264</v>
       </c>
     </row>
   </sheetData>
@@ -796,16 +796,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.7511203033436746</v>
+        <v>0.744200826183667</v>
       </c>
       <c r="C3" t="n">
-        <v>0.9011579818031431</v>
+        <v>0.9330677290836653</v>
       </c>
       <c r="D3" t="n">
-        <v>0.8193269411543523</v>
+        <v>0.8280007070885629</v>
       </c>
       <c r="E3" t="n">
-        <v>2418</v>
+        <v>2510</v>
       </c>
     </row>
     <row r="4">
@@ -815,16 +815,16 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.5282051282051282</v>
+        <v>0.569620253164557</v>
       </c>
       <c r="C4" t="n">
-        <v>0.3512361466325661</v>
+        <v>0.271356783919598</v>
       </c>
       <c r="D4" t="n">
-        <v>0.4219150025601638</v>
+        <v>0.3675970047651463</v>
       </c>
       <c r="E4" t="n">
-        <v>1173</v>
+        <v>995</v>
       </c>
     </row>
     <row r="5">
@@ -834,16 +834,16 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.5543345543345544</v>
+        <v>0.6348122866894198</v>
       </c>
       <c r="C5" t="n">
-        <v>0.4994499449944995</v>
+        <v>0.5608040201005026</v>
       </c>
       <c r="D5" t="n">
-        <v>0.5254629629629629</v>
+        <v>0.5955176093916755</v>
       </c>
       <c r="E5" t="n">
-        <v>909</v>
+        <v>995</v>
       </c>
     </row>
     <row r="6">
@@ -853,16 +853,16 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.6766666666666666</v>
+        <v>0.7044444444444444</v>
       </c>
       <c r="C6" t="n">
-        <v>0.6766666666666666</v>
+        <v>0.7044444444444444</v>
       </c>
       <c r="D6" t="n">
-        <v>0.6766666666666666</v>
+        <v>0.7044444444444444</v>
       </c>
       <c r="E6" t="n">
-        <v>0.6766666666666666</v>
+        <v>0.7044444444444444</v>
       </c>
     </row>
     <row r="7">
@@ -872,13 +872,13 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.6112199952944525</v>
+        <v>0.6495444553458812</v>
       </c>
       <c r="C7" t="n">
-        <v>0.5839480244767362</v>
+        <v>0.5884095110345887</v>
       </c>
       <c r="D7" t="n">
-        <v>0.5889016355591598</v>
+        <v>0.5970384404151282</v>
       </c>
       <c r="E7" t="n">
         <v>4500</v>
@@ -891,13 +891,13 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.6532630263910513</v>
+        <v>0.6814121001946025</v>
       </c>
       <c r="C8" t="n">
-        <v>0.6766666666666666</v>
+        <v>0.7044444444444444</v>
       </c>
       <c r="D8" t="n">
-        <v>0.6563743722328066</v>
+        <v>0.6747957368618511</v>
       </c>
       <c r="E8" t="n">
         <v>4500</v>
@@ -917,7 +917,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.6939490445859873</v>
+        <v>0.7064856711915536</v>
       </c>
     </row>
     <row r="12">
@@ -927,7 +927,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.2673588578844906</v>
+        <v>0.2251876563803169</v>
       </c>
     </row>
     <row r="13">
@@ -937,7 +937,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.3563579277864992</v>
+        <v>0.4240121580547113</v>
       </c>
     </row>
     <row r="16">
@@ -954,10 +954,10 @@
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>0.4343887005245608</v>
+        <v>0.4561461617413137</v>
       </c>
       <c r="B17" t="n">
-        <v>0.6380661407798627</v>
+        <v>0.5616222202154912</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added Train - Val - Test sets
</commit_message>
<xml_diff>
--- a/modelado/modelos/resultados/Class/BL_cla.xlsx
+++ b/modelado/modelos/resultados/Class/BL_cla.xlsx
@@ -9,6 +9,7 @@
     <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Climatology_SQA" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Climatology_HKP" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Climatology_HKP_VALIDATION" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -197,7 +198,7 @@
       <row>20</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="6296025" cy="4667250"/>
+    <ext cx="6210300" cy="4667250"/>
     <pic>
       <nvPicPr>
         <cNvPr id="2" name="Image 2" descr="Picture"/>
@@ -222,6 +223,67 @@
 </file>
 
 <file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>13</col>
+      <colOff>0</colOff>
+      <row>0</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="8096250" cy="3000375"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>13</col>
+      <colOff>0</colOff>
+      <row>20</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="6210300" cy="4667250"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="2" name="Image 2" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
@@ -588,16 +650,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.8004422332780542</v>
+        <v>0.7458745874587459</v>
       </c>
       <c r="C3" t="n">
-        <v>0.9532587228439763</v>
+        <v>0.9783549783549783</v>
       </c>
       <c r="D3" t="n">
-        <v>0.8701923076923077</v>
+        <v>0.846441947565543</v>
       </c>
       <c r="E3" t="n">
-        <v>3038</v>
+        <v>924</v>
       </c>
     </row>
     <row r="4">
@@ -607,16 +669,16 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.7123287671232876</v>
+        <v>0.8029197080291971</v>
       </c>
       <c r="C4" t="n">
-        <v>0.426812585499316</v>
+        <v>0.3819444444444444</v>
       </c>
       <c r="D4" t="n">
-        <v>0.5337895637296834</v>
+        <v>0.5176470588235295</v>
       </c>
       <c r="E4" t="n">
-        <v>731</v>
+        <v>288</v>
       </c>
     </row>
     <row r="5">
@@ -626,16 +688,16 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.7680180180180181</v>
+        <v>0.8675496688741722</v>
       </c>
       <c r="C5" t="n">
-        <v>0.466484268125855</v>
+        <v>0.4548611111111111</v>
       </c>
       <c r="D5" t="n">
-        <v>0.5804255319148937</v>
+        <v>0.5968109339407744</v>
       </c>
       <c r="E5" t="n">
-        <v>731</v>
+        <v>288</v>
       </c>
     </row>
     <row r="6">
@@ -645,16 +707,16 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.7886666666666666</v>
+        <v>0.7633333333333333</v>
       </c>
       <c r="C6" t="n">
-        <v>0.7886666666666666</v>
+        <v>0.7633333333333333</v>
       </c>
       <c r="D6" t="n">
-        <v>0.7886666666666666</v>
+        <v>0.7633333333333333</v>
       </c>
       <c r="E6" t="n">
-        <v>0.7886666666666666</v>
+        <v>0.7633333333333333</v>
       </c>
     </row>
     <row r="7">
@@ -664,16 +726,16 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.7602630061397866</v>
+        <v>0.8054479881207049</v>
       </c>
       <c r="C7" t="n">
-        <v>0.6155185254897158</v>
+        <v>0.6050535113035113</v>
       </c>
       <c r="D7" t="n">
-        <v>0.6614691344456283</v>
+        <v>0.6536333134432822</v>
       </c>
       <c r="E7" t="n">
-        <v>4500</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="8">
@@ -683,16 +745,16 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.7808615565860051</v>
+        <v>0.7801888662400344</v>
       </c>
       <c r="C8" t="n">
-        <v>0.7886666666666666</v>
+        <v>0.7633333333333333</v>
       </c>
       <c r="D8" t="n">
-        <v>0.7684745479300926</v>
+        <v>0.7353841743111209</v>
       </c>
       <c r="E8" t="n">
-        <v>4500</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="10">
@@ -709,7 +771,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.7702127659574468</v>
+        <v>0.7337662337662337</v>
       </c>
     </row>
     <row r="12">
@@ -719,7 +781,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.3640606767794632</v>
+        <v>0.3492063492063492</v>
       </c>
     </row>
     <row r="13">
@@ -729,7 +791,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.4088729016786571</v>
+        <v>0.4253246753246753</v>
       </c>
     </row>
     <row r="16">
@@ -746,10 +808,10 @@
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>0.5031794425997246</v>
+        <v>0.4914856068940228</v>
       </c>
       <c r="B17" t="n">
-        <v>0.4482800819931264</v>
+        <v>-0.02242036903412026</v>
       </c>
     </row>
   </sheetData>
@@ -796,16 +858,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.744200826183667</v>
+        <v>0.7302192564346998</v>
       </c>
       <c r="C3" t="n">
-        <v>0.9330677290836653</v>
+        <v>0.945679012345679</v>
       </c>
       <c r="D3" t="n">
-        <v>0.8280007070885629</v>
+        <v>0.8240989779451318</v>
       </c>
       <c r="E3" t="n">
-        <v>2510</v>
+        <v>810</v>
       </c>
     </row>
     <row r="4">
@@ -815,16 +877,16 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.569620253164557</v>
+        <v>0.5443037974683544</v>
       </c>
       <c r="C4" t="n">
-        <v>0.271356783919598</v>
+        <v>0.2492753623188406</v>
       </c>
       <c r="D4" t="n">
-        <v>0.3675970047651463</v>
+        <v>0.341948310139165</v>
       </c>
       <c r="E4" t="n">
-        <v>995</v>
+        <v>345</v>
       </c>
     </row>
     <row r="5">
@@ -834,16 +896,16 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.6348122866894198</v>
+        <v>0.6075085324232082</v>
       </c>
       <c r="C5" t="n">
-        <v>0.5608040201005026</v>
+        <v>0.5159420289855072</v>
       </c>
       <c r="D5" t="n">
-        <v>0.5955176093916755</v>
+        <v>0.5579937304075235</v>
       </c>
       <c r="E5" t="n">
-        <v>995</v>
+        <v>345</v>
       </c>
     </row>
     <row r="6">
@@ -853,16 +915,16 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.7044444444444444</v>
+        <v>0.6866666666666666</v>
       </c>
       <c r="C6" t="n">
-        <v>0.7044444444444444</v>
+        <v>0.6866666666666666</v>
       </c>
       <c r="D6" t="n">
-        <v>0.7044444444444444</v>
+        <v>0.6866666666666666</v>
       </c>
       <c r="E6" t="n">
-        <v>0.7044444444444444</v>
+        <v>0.6866666666666666</v>
       </c>
     </row>
     <row r="7">
@@ -872,16 +934,16 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.6495444553458812</v>
+        <v>0.6273438621087543</v>
       </c>
       <c r="C7" t="n">
-        <v>0.5884095110345887</v>
+        <v>0.5702988012166755</v>
       </c>
       <c r="D7" t="n">
-        <v>0.5970384404151282</v>
+        <v>0.5746803394972734</v>
       </c>
       <c r="E7" t="n">
-        <v>4500</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="8">
@@ -891,16 +953,16 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.6814121001946025</v>
+        <v>0.6592352343497974</v>
       </c>
       <c r="C8" t="n">
-        <v>0.7044444444444444</v>
+        <v>0.6866666666666666</v>
       </c>
       <c r="D8" t="n">
-        <v>0.6747957368618511</v>
+        <v>0.6520001174161095</v>
       </c>
       <c r="E8" t="n">
-        <v>4500</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="10">
@@ -917,7 +979,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.7064856711915536</v>
+        <v>0.7008234217749314</v>
       </c>
     </row>
     <row r="12">
@@ -927,7 +989,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.2251876563803169</v>
+        <v>0.2062350119904077</v>
       </c>
     </row>
     <row r="13">
@@ -937,7 +999,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.4240121580547113</v>
+        <v>0.3869565217391304</v>
       </c>
     </row>
     <row r="16">
@@ -954,10 +1016,218 @@
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>0.4561461617413137</v>
+        <v>0.4336052831371037</v>
       </c>
       <c r="B17" t="n">
-        <v>0.5616222202154912</v>
+        <v>0.3863702036408985</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A2:E17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="2">
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>precision</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>recall</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>f1-score</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>support</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>0.7492850333651097</v>
+      </c>
+      <c r="C3" t="n">
+        <v>0.9247058823529412</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0.8278041074249605</v>
+      </c>
+      <c r="E3" t="n">
+        <v>1700</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>0.5632911392405063</v>
+      </c>
+      <c r="C4" t="n">
+        <v>0.2738461538461539</v>
+      </c>
+      <c r="D4" t="n">
+        <v>0.3685300207039338</v>
+      </c>
+      <c r="E4" t="n">
+        <v>650</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>0.6484641638225256</v>
+      </c>
+      <c r="C5" t="n">
+        <v>0.5846153846153846</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0.6148867313915858</v>
+      </c>
+      <c r="E5" t="n">
+        <v>650</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>accuracy</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>0.71</v>
+      </c>
+      <c r="C6" t="n">
+        <v>0.71</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0.71</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0.71</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>macro avg</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>0.6536801121427138</v>
+      </c>
+      <c r="C7" t="n">
+        <v>0.5943891402714933</v>
+      </c>
+      <c r="D7" t="n">
+        <v>0.6037402865068267</v>
+      </c>
+      <c r="E7" t="n">
+        <v>3000</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>weighted avg</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>0.6871418345705524</v>
+      </c>
+      <c r="C8" t="n">
+        <v>0.71</v>
+      </c>
+      <c r="D8" t="n">
+        <v>0.6821626238281735</v>
+      </c>
+      <c r="E8" t="n">
+        <v>3000</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>IoU</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Class 0</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>0.706199460916442</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Class 1</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>0.2258883248730965</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Class 2</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>0.4439252336448598</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>Cohen's Kappa</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Aggregated R2</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>0.4615337005632234</v>
+      </c>
+      <c r="B17" t="n">
+        <v>0.6392909280500522</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Diagrams and changed vars
</commit_message>
<xml_diff>
--- a/modelado/modelos/resultados/Class/BL_cla.xlsx
+++ b/modelado/modelos/resultados/Class/BL_cla.xlsx
@@ -10,6 +10,7 @@
     <sheet name="Climatology_SQA" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Climatology_HKP" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Climatology_HKP_VALIDATION" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Climatology_SQA_VALIDATION" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -284,6 +285,67 @@
 </file>
 
 <file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>13</col>
+      <colOff>0</colOff>
+      <row>0</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="8096250" cy="3000375"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>13</col>
+      <colOff>0</colOff>
+      <row>20</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="6296025" cy="4667250"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="2" name="Image 2" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
@@ -650,13 +712,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.7458745874587459</v>
+        <v>0.7475165562913907</v>
       </c>
       <c r="C3" t="n">
-        <v>0.9783549783549783</v>
+        <v>0.9772727272727273</v>
       </c>
       <c r="D3" t="n">
-        <v>0.846441947565543</v>
+        <v>0.8470919324577861</v>
       </c>
       <c r="E3" t="n">
         <v>924</v>
@@ -669,13 +731,13 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.8029197080291971</v>
+        <v>0.7876712328767124</v>
       </c>
       <c r="C4" t="n">
-        <v>0.3819444444444444</v>
+        <v>0.3993055555555556</v>
       </c>
       <c r="D4" t="n">
-        <v>0.5176470588235295</v>
+        <v>0.5299539170506913</v>
       </c>
       <c r="E4" t="n">
         <v>288</v>
@@ -688,13 +750,13 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.8675496688741722</v>
+        <v>0.8698630136986302</v>
       </c>
       <c r="C5" t="n">
-        <v>0.4548611111111111</v>
+        <v>0.4409722222222222</v>
       </c>
       <c r="D5" t="n">
-        <v>0.5968109339407744</v>
+        <v>0.5852534562211982</v>
       </c>
       <c r="E5" t="n">
         <v>288</v>
@@ -726,13 +788,13 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.8054479881207049</v>
+        <v>0.8016836009555778</v>
       </c>
       <c r="C7" t="n">
-        <v>0.6050535113035113</v>
+        <v>0.6058501683501684</v>
       </c>
       <c r="D7" t="n">
-        <v>0.6536333134432822</v>
+        <v>0.6540997685765585</v>
       </c>
       <c r="E7" t="n">
         <v>1500</v>
@@ -745,13 +807,13 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.7801888662400344</v>
+        <v>0.7787167740179624</v>
       </c>
       <c r="C8" t="n">
         <v>0.7633333333333333</v>
       </c>
       <c r="D8" t="n">
-        <v>0.7353841743111209</v>
+        <v>0.735928446062199</v>
       </c>
       <c r="E8" t="n">
         <v>1500</v>
@@ -771,7 +833,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.7337662337662337</v>
+        <v>0.7347436940602116</v>
       </c>
     </row>
     <row r="12">
@@ -781,7 +843,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.3492063492063492</v>
+        <v>0.3605015673981191</v>
       </c>
     </row>
     <row r="13">
@@ -791,7 +853,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.4253246753246753</v>
+        <v>0.4136807817589577</v>
       </c>
     </row>
     <row r="16">
@@ -808,10 +870,10 @@
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>0.4914856068940228</v>
+        <v>0.492718002652156</v>
       </c>
       <c r="B17" t="n">
-        <v>-0.02242036903412026</v>
+        <v>-0.02381197814658287</v>
       </c>
     </row>
   </sheetData>
@@ -1234,4 +1296,212 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A2:E17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="2">
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>precision</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>recall</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>f1-score</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>support</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>0.8249172185430463</v>
+      </c>
+      <c r="C3" t="n">
+        <v>0.9427625354777672</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0.8799116997792494</v>
+      </c>
+      <c r="E3" t="n">
+        <v>2114</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>0.6746575342465754</v>
+      </c>
+      <c r="C4" t="n">
+        <v>0.4446952595936794</v>
+      </c>
+      <c r="D4" t="n">
+        <v>0.5360544217687074</v>
+      </c>
+      <c r="E4" t="n">
+        <v>443</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>0.7157534246575342</v>
+      </c>
+      <c r="C5" t="n">
+        <v>0.4717832957110609</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0.5687074829931973</v>
+      </c>
+      <c r="E5" t="n">
+        <v>443</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>accuracy</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>0.7996666666666666</v>
+      </c>
+      <c r="C6" t="n">
+        <v>0.7996666666666666</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0.7996666666666666</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0.7996666666666666</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>macro avg</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>0.7384427258157187</v>
+      </c>
+      <c r="C7" t="n">
+        <v>0.6197470302608359</v>
+      </c>
+      <c r="D7" t="n">
+        <v>0.6615578681803848</v>
+      </c>
+      <c r="E7" t="n">
+        <v>3000</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>weighted avg</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>0.7866090182648401</v>
+      </c>
+      <c r="C8" t="n">
+        <v>0.7996666666666666</v>
+      </c>
+      <c r="D8" t="n">
+        <v>0.7831809523809523</v>
+      </c>
+      <c r="E8" t="n">
+        <v>3000</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>IoU</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Class 0</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>0.7855735120220733</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Class 1</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>0.3661710037174721</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Class 2</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>0.3973384030418251</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>Cohen's Kappa</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Aggregated R2</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>0.5038339354472264</v>
+      </c>
+      <c r="B17" t="n">
+        <v>0.5877690239434619</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Refactor and increase prediction horizont
</commit_message>
<xml_diff>
--- a/modelado/modelos/resultados/Class/BL_cla.xlsx
+++ b/modelado/modelos/resultados/Class/BL_cla.xlsx
@@ -474,13 +474,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.7475165562913907</v>
+        <v>0.7685738684884714</v>
       </c>
       <c r="C3" t="n">
-        <v>0.9772727272727273</v>
+        <v>0.974025974025974</v>
       </c>
       <c r="D3" t="n">
-        <v>0.8470919324577861</v>
+        <v>0.8591885441527446</v>
       </c>
       <c r="E3" t="n">
         <v>924</v>
@@ -493,13 +493,13 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.7876712328767124</v>
+        <v>0.7777777777777778</v>
       </c>
       <c r="C4" t="n">
-        <v>0.3993055555555556</v>
+        <v>0.4375</v>
       </c>
       <c r="D4" t="n">
-        <v>0.5299539170506913</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="E4" t="n">
         <v>288</v>
@@ -512,13 +512,13 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.8698630136986302</v>
+        <v>0.8682634730538922</v>
       </c>
       <c r="C5" t="n">
-        <v>0.4409722222222222</v>
+        <v>0.5034722222222222</v>
       </c>
       <c r="D5" t="n">
-        <v>0.5852534562211982</v>
+        <v>0.6373626373626373</v>
       </c>
       <c r="E5" t="n">
         <v>288</v>
@@ -531,16 +531,16 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.7633333333333333</v>
+        <v>0.7806666666666666</v>
       </c>
       <c r="C6" t="n">
-        <v>0.7633333333333333</v>
+        <v>0.7806666666666666</v>
       </c>
       <c r="D6" t="n">
-        <v>0.7633333333333333</v>
+        <v>0.7806666666666666</v>
       </c>
       <c r="E6" t="n">
-        <v>0.7633333333333333</v>
+        <v>0.7806666666666666</v>
       </c>
     </row>
     <row r="7">
@@ -550,13 +550,13 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.8016836009555778</v>
+        <v>0.8048717064400471</v>
       </c>
       <c r="C7" t="n">
-        <v>0.6058501683501684</v>
+        <v>0.638332732082732</v>
       </c>
       <c r="D7" t="n">
-        <v>0.6540997685765585</v>
+        <v>0.6855170605051274</v>
       </c>
       <c r="E7" t="n">
         <v>1500</v>
@@ -569,13 +569,13 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.7787167740179624</v>
+        <v>0.7894814231485791</v>
       </c>
       <c r="C8" t="n">
-        <v>0.7633333333333333</v>
+        <v>0.7806666666666666</v>
       </c>
       <c r="D8" t="n">
-        <v>0.735928446062199</v>
+        <v>0.759153769571717</v>
       </c>
       <c r="E8" t="n">
         <v>1500</v>
@@ -595,7 +595,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.7347436940602116</v>
+        <v>0.7531380753138075</v>
       </c>
     </row>
     <row r="12">
@@ -605,7 +605,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.3605015673981191</v>
+        <v>0.3888888888888889</v>
       </c>
     </row>
     <row r="13">
@@ -615,7 +615,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.4136807817589577</v>
+        <v>0.4677419354838709</v>
       </c>
     </row>
     <row r="16">
@@ -624,18 +624,10 @@
           <t>Cohen's Kappa</t>
         </is>
       </c>
-      <c r="B16" s="2" t="inlineStr">
-        <is>
-          <t>Aggregated R2</t>
-        </is>
-      </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>0.492718002652156</v>
-      </c>
-      <c r="B17" t="n">
-        <v>-0.02381197814658287</v>
+        <v>0.5401791204982278</v>
       </c>
     </row>
   </sheetData>
@@ -681,13 +673,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.7302192564346998</v>
+        <v>0.7456479690522244</v>
       </c>
       <c r="C3" t="n">
-        <v>0.945679012345679</v>
+        <v>0.9518518518518518</v>
       </c>
       <c r="D3" t="n">
-        <v>0.8240989779451318</v>
+        <v>0.8362255965292842</v>
       </c>
       <c r="E3" t="n">
         <v>810</v>
@@ -700,13 +692,13 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.5443037974683544</v>
+        <v>0.5426829268292683</v>
       </c>
       <c r="C4" t="n">
-        <v>0.2492753623188406</v>
+        <v>0.2579710144927536</v>
       </c>
       <c r="D4" t="n">
-        <v>0.341948310139165</v>
+        <v>0.3497053045186641</v>
       </c>
       <c r="E4" t="n">
         <v>345</v>
@@ -719,13 +711,13 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.6075085324232082</v>
+        <v>0.5960264900662252</v>
       </c>
       <c r="C5" t="n">
-        <v>0.5159420289855072</v>
+        <v>0.5217391304347826</v>
       </c>
       <c r="D5" t="n">
-        <v>0.5579937304075235</v>
+        <v>0.5564142194744977</v>
       </c>
       <c r="E5" t="n">
         <v>345</v>
@@ -738,16 +730,16 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.6866666666666666</v>
+        <v>0.6933333333333334</v>
       </c>
       <c r="C6" t="n">
-        <v>0.6866666666666666</v>
+        <v>0.6933333333333334</v>
       </c>
       <c r="D6" t="n">
-        <v>0.6866666666666666</v>
+        <v>0.6933333333333334</v>
       </c>
       <c r="E6" t="n">
-        <v>0.6866666666666666</v>
+        <v>0.6933333333333334</v>
       </c>
     </row>
     <row r="7">
@@ -757,13 +749,13 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.6273438621087543</v>
+        <v>0.6281191286492392</v>
       </c>
       <c r="C7" t="n">
-        <v>0.5702988012166755</v>
+        <v>0.577187332259796</v>
       </c>
       <c r="D7" t="n">
-        <v>0.5746803394972734</v>
+        <v>0.5807817068408153</v>
       </c>
       <c r="E7" t="n">
         <v>1500</v>
@@ -776,13 +768,13 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.6592352343497974</v>
+        <v>0.6645530691741647</v>
       </c>
       <c r="C8" t="n">
-        <v>0.6866666666666666</v>
+        <v>0.6933333333333334</v>
       </c>
       <c r="D8" t="n">
-        <v>0.6520001174161095</v>
+        <v>0.6599693126442406</v>
       </c>
       <c r="E8" t="n">
         <v>1500</v>
@@ -802,7 +794,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.7008234217749314</v>
+        <v>0.7185461323392358</v>
       </c>
     </row>
     <row r="12">
@@ -812,7 +804,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.2062350119904077</v>
+        <v>0.2119047619047619</v>
       </c>
     </row>
     <row r="13">
@@ -822,7 +814,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.3869565217391304</v>
+        <v>0.3854389721627409</v>
       </c>
     </row>
     <row r="16">
@@ -831,18 +823,10 @@
           <t>Cohen's Kappa</t>
         </is>
       </c>
-      <c r="B16" s="2" t="inlineStr">
-        <is>
-          <t>Aggregated R2</t>
-        </is>
-      </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>0.4336052831371037</v>
-      </c>
-      <c r="B17" t="n">
-        <v>0.3863702036408985</v>
+        <v>0.4487452963593223</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
pred de anomalias y percentiles
</commit_message>
<xml_diff>
--- a/modelado/modelos/resultados/Class/BL_cla.xlsx
+++ b/modelado/modelos/resultados/Class/BL_cla.xlsx
@@ -474,13 +474,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.7685738684884714</v>
+        <v>0.7670648464163823</v>
       </c>
       <c r="C3" t="n">
-        <v>0.974025974025974</v>
+        <v>0.9729437229437229</v>
       </c>
       <c r="D3" t="n">
-        <v>0.8591885441527446</v>
+        <v>0.857824427480916</v>
       </c>
       <c r="E3" t="n">
         <v>924</v>
@@ -493,16 +493,16 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.7777777777777778</v>
+        <v>0.8577586206896551</v>
       </c>
       <c r="C4" t="n">
-        <v>0.4375</v>
+        <v>0.4937965260545906</v>
       </c>
       <c r="D4" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.6267716535433071</v>
       </c>
       <c r="E4" t="n">
-        <v>288</v>
+        <v>403</v>
       </c>
     </row>
     <row r="5">
@@ -512,16 +512,16 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.8682634730538922</v>
+        <v>0.71875</v>
       </c>
       <c r="C5" t="n">
-        <v>0.5034722222222222</v>
+        <v>0.3988439306358382</v>
       </c>
       <c r="D5" t="n">
-        <v>0.6373626373626373</v>
+        <v>0.5130111524163569</v>
       </c>
       <c r="E5" t="n">
-        <v>288</v>
+        <v>173</v>
       </c>
     </row>
     <row r="6">
@@ -531,16 +531,16 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.7806666666666666</v>
+        <v>0.778</v>
       </c>
       <c r="C6" t="n">
-        <v>0.7806666666666666</v>
+        <v>0.778</v>
       </c>
       <c r="D6" t="n">
-        <v>0.7806666666666666</v>
+        <v>0.778</v>
       </c>
       <c r="E6" t="n">
-        <v>0.7806666666666666</v>
+        <v>0.778</v>
       </c>
     </row>
     <row r="7">
@@ -550,13 +550,13 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.8048717064400471</v>
+        <v>0.7811911557020125</v>
       </c>
       <c r="C7" t="n">
-        <v>0.638332732082732</v>
+        <v>0.6218613932113839</v>
       </c>
       <c r="D7" t="n">
-        <v>0.6855170605051274</v>
+        <v>0.6658690778135267</v>
       </c>
       <c r="E7" t="n">
         <v>1500</v>
@@ -569,13 +569,13 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.7894814231485791</v>
+        <v>0.7858589281511122</v>
       </c>
       <c r="C8" t="n">
-        <v>0.7806666666666666</v>
+        <v>0.778</v>
       </c>
       <c r="D8" t="n">
-        <v>0.759153769571717</v>
+        <v>0.7559797844922326</v>
       </c>
       <c r="E8" t="n">
         <v>1500</v>
@@ -595,7 +595,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.7531380753138075</v>
+        <v>0.7510442773600668</v>
       </c>
     </row>
     <row r="12">
@@ -605,7 +605,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.3888888888888889</v>
+        <v>0.4564220183486238</v>
       </c>
     </row>
     <row r="13">
@@ -615,7 +615,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.4677419354838709</v>
+        <v>0.345</v>
       </c>
     </row>
     <row r="16">
@@ -627,7 +627,7 @@
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>0.5401791204982278</v>
+        <v>0.5274218330167044</v>
       </c>
     </row>
   </sheetData>

</xml_diff>